<commit_message>
Daily Thornton Place tracker update - 2026-08-12
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="mmm\ yyyy"/>
     <numFmt numFmtId="165" formatCode="mmm\ d&quot;, &quot;yyyy"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
@@ -27,6 +27,7 @@
     <numFmt numFmtId="171" formatCode="mmm\ d"/>
     <numFmt numFmtId="172" formatCode="mmm\ dd"/>
     <numFmt numFmtId="173" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="174" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -707,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BL40"/>
+  <dimension ref="A1:BM41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -916,12 +917,15 @@
       <c r="BJ1" s="56" t="n">
         <v>46242</v>
       </c>
-      <c r="BK1" s="44" t="inlineStr">
+      <c r="BK1" s="56" t="n">
+        <v>46246.06425153022</v>
+      </c>
+      <c r="BL1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BL1" s="44" t="inlineStr">
+      <c r="BM1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -975,12 +979,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BK2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL2" s="58" t="inlineStr">
+      <c r="BL2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1034,12 +1038,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BK3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL3" s="58" t="inlineStr">
+      <c r="BL3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1094,12 +1098,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BK4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BL4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1164,12 +1168,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BK5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BL5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1229,12 +1233,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BK6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BL6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1269,7 +1273,11 @@
           <t>Available Now</t>
         </is>
       </c>
-      <c r="H7" s="42" t="n"/>
+      <c r="H7" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="AK7" s="42" t="n">
         <v>3245.06</v>
       </c>
@@ -1285,12 +1293,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BK7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BL7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1367,12 +1375,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BK8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BL8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1420,12 +1428,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BK9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BL9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1469,12 +1477,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BK10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BL10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1517,106 +1525,71 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BK11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BL11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="BM11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="43">
-      <c r="A12" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B12" s="42" t="n"/>
-      <c r="C12" s="42" t="n"/>
-      <c r="D12" s="42" t="n"/>
-      <c r="E12" s="42" t="n"/>
-      <c r="F12" s="42" t="n"/>
-      <c r="G12" s="42" t="n"/>
-      <c r="H12" s="42" t="n"/>
-      <c r="AH12" s="42" t="n"/>
-      <c r="AJ12" s="42" t="n"/>
-      <c r="AN12" s="42" t="n"/>
-      <c r="AP12" s="42" t="n"/>
-      <c r="BK12" s="42" t="n"/>
-      <c r="BL12" s="42" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>#6-481</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>605</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Sep 14</t>
+        </is>
+      </c>
+      <c r="BK12" t="n">
+        <v>2064.06</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
       <c r="A13" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B13" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C13" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E13" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F13" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G13" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H13" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z13" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB13" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE13" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG13" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ13" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="BK13" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL13" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="42" t="n"/>
+      <c r="D13" s="42" t="n"/>
+      <c r="E13" s="42" t="n"/>
+      <c r="F13" s="42" t="n"/>
+      <c r="G13" s="42" t="n"/>
+      <c r="H13" s="42" t="n"/>
+      <c r="AH13" s="42" t="n"/>
+      <c r="AJ13" s="42" t="n"/>
+      <c r="AN13" s="42" t="n"/>
+      <c r="AP13" s="42" t="n"/>
+      <c r="BL13" s="42" t="n"/>
+      <c r="BM13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B14" s="42" t="inlineStr">
@@ -1626,25 +1599,25 @@
       </c>
       <c r="C14" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D14" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E14" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F14" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G14" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H14" s="42" t="inlineStr">
@@ -1652,21 +1625,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF14" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z14" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB14" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE14" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG14" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI14" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="BK14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ14" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="BL14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1675,606 +1654,670 @@
     <row r="15" ht="15.75" customHeight="1" s="43">
       <c r="A15" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C15" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E15" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F15" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G15" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H15" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF15" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG15" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI15" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="BL15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1" s="43">
+      <c r="A16" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C15" s="42" t="inlineStr">
+      <c r="C16" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D15" s="42" t="inlineStr">
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E15" s="42" t="n">
+      <c r="E16" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F15" s="42" t="inlineStr">
+      <c r="F16" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G15" s="42" t="inlineStr">
+      <c r="G16" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H15" s="42" t="inlineStr">
+      <c r="H16" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I15" s="42" t="n">
+      <c r="I16" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J15" s="42" t="n">
+      <c r="J16" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K15" s="42" t="n">
+      <c r="K16" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L15" s="42" t="n">
+      <c r="L16" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N15" s="42" t="n">
+      <c r="N16" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O15" s="42" t="n">
+      <c r="O16" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q15" s="42" t="n">
+      <c r="Q16" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T15" s="42" t="n">
+      <c r="T16" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U15" s="42" t="n">
+      <c r="U16" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V15" s="42" t="n">
+      <c r="V16" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W15" s="42" t="n">
+      <c r="W16" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA15" s="42" t="n">
+      <c r="AA16" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB15" s="42" t="n">
+      <c r="AB16" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC15" s="42" t="n">
+      <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BK15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL15" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15.75" customHeight="1" s="43">
-      <c r="A16" s="61" t="inlineStr">
+      <c r="BL16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM16" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1" s="43">
+      <c r="A17" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B16" s="62" t="inlineStr">
+      <c r="B17" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C16" s="61" t="inlineStr">
+      <c r="C17" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D16" s="61" t="inlineStr">
+      <c r="D17" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E16" s="63" t="n">
+      <c r="E17" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F16" s="64" t="inlineStr">
+      <c r="F17" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G16" s="64" t="inlineStr">
+      <c r="G17" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H16" s="65" t="inlineStr">
+      <c r="H17" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I16" s="66" t="n">
+      <c r="I17" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J16" s="67" t="n">
+      <c r="J17" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K16" s="66" t="n">
+      <c r="K17" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L16" s="68" t="n">
+      <c r="L17" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M16" s="68" t="n"/>
-      <c r="N16" s="69" t="n">
+      <c r="M17" s="68" t="n"/>
+      <c r="N17" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O16" s="69" t="n">
+      <c r="O17" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q16" s="42" t="n">
+      <c r="Q17" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T16" s="42" t="n">
+      <c r="T17" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U16" s="42" t="n">
+      <c r="U17" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V16" s="42" t="n">
+      <c r="V17" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W16" s="42" t="n">
+      <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BK16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL16" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15.75" customHeight="1" s="43">
-      <c r="A17" s="42" t="inlineStr">
+      <c r="BL17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM17" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" s="43">
+      <c r="A18" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B17" s="42" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C17" s="42" t="inlineStr">
+      <c r="C18" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E17" s="42" t="n">
+      <c r="E18" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F17" s="42" t="inlineStr">
+      <c r="F18" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G17" s="42" t="inlineStr">
+      <c r="G18" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H17" s="42" t="inlineStr">
+      <c r="H18" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I17" s="42" t="n">
+      <c r="I18" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M17" s="42" t="n">
+      <c r="M18" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N17" s="42" t="n">
+      <c r="N18" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q17" s="42" t="n">
+      <c r="Q18" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V17" s="42" t="n">
+      <c r="V18" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W17" s="42" t="n">
+      <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BK17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL17" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" s="43">
-      <c r="A18" s="61" t="inlineStr">
+      <c r="BL18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM18" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1" s="43">
+      <c r="A19" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B18" s="62" t="inlineStr">
+      <c r="B19" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C18" s="61" t="inlineStr">
+      <c r="C19" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D18" s="61" t="inlineStr">
+      <c r="D19" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E18" s="63" t="n">
+      <c r="E19" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F18" s="64" t="inlineStr">
+      <c r="F19" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G18" s="64" t="inlineStr">
+      <c r="G19" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H18" s="65" t="inlineStr">
+      <c r="H19" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I18" s="66" t="n">
+      <c r="I19" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J18" s="67" t="n">
+      <c r="J19" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K18" s="66" t="n">
+      <c r="K19" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L18" s="68" t="n">
+      <c r="L19" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M18" s="68" t="n"/>
-      <c r="N18" s="69" t="n">
+      <c r="M19" s="68" t="n"/>
+      <c r="N19" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O18" s="69" t="n">
+      <c r="O19" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q18" s="42" t="n">
+      <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BK18" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL18" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="43">
-      <c r="A19" s="42" t="inlineStr">
+      <c r="BL19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM19" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="43">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B20" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C20" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D19" s="42" t="inlineStr">
+      <c r="D20" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E19" s="42" t="n">
+      <c r="E20" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F19" s="42" t="inlineStr">
+      <c r="F20" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G19" s="42" t="inlineStr">
+      <c r="G20" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H19" s="42" t="inlineStr">
+      <c r="H20" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I19" s="72" t="n">
+      <c r="I20" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J19" s="72" t="n">
+      <c r="J20" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K19" s="72" t="n">
+      <c r="K20" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L19" s="72" t="n">
+      <c r="L20" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M19" s="72" t="n"/>
-      <c r="N19" s="42" t="n">
+      <c r="M20" s="72" t="n"/>
+      <c r="N20" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O19" s="42" t="n">
+      <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BK19" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL19" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="43">
-      <c r="A20" s="61" t="inlineStr">
+      <c r="BL20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM20" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="43">
+      <c r="A21" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B20" s="62" t="inlineStr">
+      <c r="B21" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C20" s="61" t="inlineStr">
+      <c r="C21" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D20" s="61" t="inlineStr">
+      <c r="D21" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E20" s="64" t="n">
+      <c r="E21" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F20" s="64" t="inlineStr">
+      <c r="F21" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G20" s="73" t="n">
+      <c r="G21" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H20" s="65" t="inlineStr">
+      <c r="H21" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I20" s="66" t="n">
+      <c r="I21" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J20" s="66" t="n">
+      <c r="J21" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K20" s="67" t="n">
+      <c r="K21" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L20" s="68" t="n">
+      <c r="L21" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M20" s="68" t="n"/>
-      <c r="N20" s="69" t="n">
+      <c r="M21" s="68" t="n"/>
+      <c r="N21" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O20" s="69" t="n"/>
-      <c r="BK20" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL20" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="43">
-      <c r="A21" s="75" t="inlineStr">
+      <c r="O21" s="69" t="n"/>
+      <c r="BL21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM21" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="43">
+      <c r="A22" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B21" s="76" t="inlineStr">
+      <c r="B22" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C21" s="75" t="inlineStr">
+      <c r="C22" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D21" s="75" t="inlineStr">
+      <c r="D22" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E21" s="77" t="n">
+      <c r="E22" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F21" s="78" t="inlineStr">
+      <c r="F22" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G21" s="79" t="n">
+      <c r="G22" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H21" s="80" t="inlineStr">
+      <c r="H22" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I21" s="81" t="n">
+      <c r="I22" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J21" s="81" t="n">
+      <c r="J22" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K21" s="82" t="inlineStr">
+      <c r="K22" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L21" s="83" t="inlineStr">
+      <c r="L22" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M21" s="83" t="n"/>
-      <c r="N21" s="84" t="n"/>
-      <c r="O21" s="69" t="n"/>
-      <c r="BK21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL21" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="43">
-      <c r="A22" s="42" t="inlineStr">
+      <c r="M22" s="83" t="n"/>
+      <c r="N22" s="84" t="n"/>
+      <c r="O22" s="69" t="n"/>
+      <c r="BL22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM22" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="43">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B23" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C23" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D22" s="42" t="inlineStr">
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E22" s="42" t="n">
+      <c r="E23" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F22" s="42" t="inlineStr">
+      <c r="F23" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G22" s="47" t="n">
+      <c r="G23" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H22" s="42" t="inlineStr">
+      <c r="H23" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I22" s="72" t="n">
+      <c r="I23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J22" s="72" t="n">
+      <c r="J23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K22" s="72" t="n">
+      <c r="K23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L22" s="72" t="n">
+      <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BK22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BL22" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="43"/>
+      <c r="BL23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BM23" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="24" ht="15.75" customHeight="1" s="43"/>
     <row r="25" ht="15.75" customHeight="1" s="43"/>
     <row r="26" ht="15.75" customHeight="1" s="43"/>
     <row r="27" ht="15.75" customHeight="1" s="43"/>
     <row r="28" ht="15.75" customHeight="1" s="43"/>
-    <row r="31" ht="15.75" customHeight="1" s="43">
-      <c r="A31" s="42" t="n"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" s="43">
-      <c r="A34" s="42" t="n"/>
-    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31" ht="15.75" customHeight="1" s="43"/>
+    <row r="32">
+      <c r="A32" s="42" t="n"/>
+    </row>
+    <row r="33"/>
+    <row r="34" ht="15.75" customHeight="1" s="43"/>
     <row r="35" ht="15.75" customHeight="1" s="43">
       <c r="A35" s="42" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="43">
       <c r="A36" s="42" t="n"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1" s="43">
-      <c r="A38" s="42" t="n"/>
-    </row>
+    <row r="37">
+      <c r="A37" s="42" t="n"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" s="43"/>
     <row r="39" ht="15.75" customHeight="1" s="43">
       <c r="A39" s="42" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="43">
       <c r="A40" s="42" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-13
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BN41"/>
+  <dimension ref="A1:BO41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -921,14 +921,17 @@
         <v>46246.06425152778</v>
       </c>
       <c r="BL1" s="56" t="n">
-        <v>46246.59625842162</v>
-      </c>
-      <c r="BM1" s="44" t="inlineStr">
+        <v>46246.59625842593</v>
+      </c>
+      <c r="BM1" s="56" t="n">
+        <v>46247.59313046772</v>
+      </c>
+      <c r="BN1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BN1" s="44" t="inlineStr">
+      <c r="BO1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -982,12 +985,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BM2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN2" s="58" t="inlineStr">
+      <c r="BN2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1041,12 +1044,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BM3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN3" s="58" t="inlineStr">
+      <c r="BN3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1101,12 +1104,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BM4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1171,12 +1174,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BM5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1236,12 +1239,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BM6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1296,12 +1299,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BM7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1378,12 +1381,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BM8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1431,12 +1434,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BM9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1480,12 +1483,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BM10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1528,12 +1531,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BM11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1586,8 +1589,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BM13" s="42" t="n"/>
       <c r="BN13" s="42" t="n"/>
+      <c r="BO13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1643,12 +1646,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BM14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN14" s="58" t="inlineStr">
+      <c r="BN14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1702,12 +1705,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BM15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BN15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1794,12 +1797,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BM16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN16" s="58" t="inlineStr">
+      <c r="BN16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1878,12 +1881,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BM17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN17" s="58" t="inlineStr">
+      <c r="BN17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1946,12 +1949,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BM18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN18" s="58" t="inlineStr">
+      <c r="BN18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2018,12 +2021,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BM19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN19" s="71" t="inlineStr">
+      <c r="BN19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2087,12 +2090,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BM20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN20" s="58" t="inlineStr">
+      <c r="BN20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2152,12 +2155,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BM21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN21" s="71" t="inlineStr">
+      <c r="BN21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2219,12 +2222,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BM22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN22" s="71" t="inlineStr">
+      <c r="BN22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2279,12 +2282,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BM23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BN23" s="58" t="inlineStr">
+      <c r="BN23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BO23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-15
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BO41"/>
+  <dimension ref="A1:BP41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -924,14 +924,17 @@
         <v>46246.59625842593</v>
       </c>
       <c r="BM1" s="56" t="n">
-        <v>46247.59313046772</v>
-      </c>
-      <c r="BN1" s="44" t="inlineStr">
+        <v>46247.59313046296</v>
+      </c>
+      <c r="BN1" s="56" t="n">
+        <v>46249.56688524211</v>
+      </c>
+      <c r="BO1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BO1" s="44" t="inlineStr">
+      <c r="BP1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -985,12 +988,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BN2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO2" s="58" t="inlineStr">
+      <c r="BO2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1044,12 +1047,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BN3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO3" s="58" t="inlineStr">
+      <c r="BO3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1104,12 +1107,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BN4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1174,12 +1177,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BN5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1239,12 +1242,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BN6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1299,12 +1302,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BN7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1381,12 +1384,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BN8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1434,12 +1437,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BN9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1479,16 +1482,20 @@
           <t>Sep 28</t>
         </is>
       </c>
-      <c r="H10" s="42" t="n"/>
+      <c r="H10" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BN10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1531,12 +1538,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BN11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1589,8 +1596,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BN13" s="42" t="n"/>
       <c r="BO13" s="42" t="n"/>
+      <c r="BP13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1646,12 +1653,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BN14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO14" s="58" t="inlineStr">
+      <c r="BO14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1705,12 +1712,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BN15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BO15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1797,12 +1804,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BN16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO16" s="58" t="inlineStr">
+      <c r="BO16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1881,12 +1888,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BN17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO17" s="58" t="inlineStr">
+      <c r="BO17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1949,12 +1956,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BN18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO18" s="58" t="inlineStr">
+      <c r="BO18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2021,12 +2028,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BN19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO19" s="71" t="inlineStr">
+      <c r="BO19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2090,12 +2097,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BN20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO20" s="58" t="inlineStr">
+      <c r="BO20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2155,12 +2162,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BN21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO21" s="71" t="inlineStr">
+      <c r="BO21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2222,12 +2229,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BN22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO22" s="71" t="inlineStr">
+      <c r="BO22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2282,12 +2289,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BN23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BO23" s="58" t="inlineStr">
+      <c r="BO23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BP23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-16
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BP41"/>
+  <dimension ref="A1:BQ41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -927,14 +927,17 @@
         <v>46247.59313046296</v>
       </c>
       <c r="BN1" s="56" t="n">
-        <v>46249.56688524211</v>
-      </c>
-      <c r="BO1" s="44" t="inlineStr">
+        <v>46249.56688524305</v>
+      </c>
+      <c r="BO1" s="56" t="n">
+        <v>46250.56750208638</v>
+      </c>
+      <c r="BP1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BP1" s="44" t="inlineStr">
+      <c r="BQ1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -988,12 +991,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BO2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP2" s="58" t="inlineStr">
+      <c r="BP2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1047,12 +1050,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BO3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP3" s="58" t="inlineStr">
+      <c r="BP3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1107,12 +1110,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BO4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1177,12 +1180,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BO5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1242,12 +1245,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BO6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1302,12 +1305,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BO7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1384,12 +1387,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BO8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1437,12 +1440,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BO9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1490,12 +1493,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BO10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1538,12 +1541,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BO11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1596,8 +1599,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BO13" s="42" t="n"/>
       <c r="BP13" s="42" t="n"/>
+      <c r="BQ13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1653,12 +1656,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BO14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP14" s="58" t="inlineStr">
+      <c r="BP14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1712,12 +1715,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BO15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BP15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1804,12 +1807,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BO16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP16" s="58" t="inlineStr">
+      <c r="BP16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1888,12 +1891,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BO17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP17" s="58" t="inlineStr">
+      <c r="BP17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1956,12 +1959,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BO18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP18" s="58" t="inlineStr">
+      <c r="BP18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2028,12 +2031,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BO19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP19" s="71" t="inlineStr">
+      <c r="BP19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2097,12 +2100,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BO20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP20" s="58" t="inlineStr">
+      <c r="BP20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2162,12 +2165,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BO21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP21" s="71" t="inlineStr">
+      <c r="BP21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2229,12 +2232,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BO22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP22" s="71" t="inlineStr">
+      <c r="BP22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2289,12 +2292,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BO23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BP23" s="58" t="inlineStr">
+      <c r="BP23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BQ23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-17
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BQ41"/>
+  <dimension ref="A1:BR41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -930,14 +930,17 @@
         <v>46249.56688524305</v>
       </c>
       <c r="BO1" s="56" t="n">
-        <v>46250.56750208638</v>
-      </c>
-      <c r="BP1" s="44" t="inlineStr">
+        <v>46250.56750208334</v>
+      </c>
+      <c r="BP1" s="56" t="n">
+        <v>46251.5730979497</v>
+      </c>
+      <c r="BQ1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BQ1" s="44" t="inlineStr">
+      <c r="BR1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -991,12 +994,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BP2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ2" s="58" t="inlineStr">
+      <c r="BQ2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1050,12 +1053,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BP3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ3" s="58" t="inlineStr">
+      <c r="BQ3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1110,12 +1113,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BP4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1180,12 +1183,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BP5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1245,12 +1248,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BP6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1305,12 +1308,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BP7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1387,12 +1390,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BP8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1440,12 +1443,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BP9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1493,12 +1496,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BP10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1541,12 +1544,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BP11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1599,8 +1602,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BP13" s="42" t="n"/>
       <c r="BQ13" s="42" t="n"/>
+      <c r="BR13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1656,12 +1659,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BP14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ14" s="58" t="inlineStr">
+      <c r="BQ14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1715,12 +1718,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BP15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BQ15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1807,12 +1810,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BP16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ16" s="58" t="inlineStr">
+      <c r="BQ16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1891,12 +1894,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BP17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ17" s="58" t="inlineStr">
+      <c r="BQ17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1959,12 +1962,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BP18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ18" s="58" t="inlineStr">
+      <c r="BQ18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2031,12 +2034,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BP19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ19" s="71" t="inlineStr">
+      <c r="BQ19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2100,12 +2103,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BP20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ20" s="58" t="inlineStr">
+      <c r="BQ20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2165,12 +2168,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BP21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ21" s="71" t="inlineStr">
+      <c r="BQ21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2232,12 +2235,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BP22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ22" s="71" t="inlineStr">
+      <c r="BQ22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2292,12 +2295,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BP23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BQ23" s="58" t="inlineStr">
+      <c r="BQ23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BR23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-18
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BR41"/>
+  <dimension ref="A1:BS41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -933,14 +933,17 @@
         <v>46250.56750208334</v>
       </c>
       <c r="BP1" s="56" t="n">
-        <v>46251.5730979497</v>
-      </c>
-      <c r="BQ1" s="44" t="inlineStr">
+        <v>46251.57309795139</v>
+      </c>
+      <c r="BQ1" s="56" t="n">
+        <v>46252.57610714522</v>
+      </c>
+      <c r="BR1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BR1" s="44" t="inlineStr">
+      <c r="BS1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -994,12 +997,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BQ2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR2" s="58" t="inlineStr">
+      <c r="BR2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1053,12 +1056,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BQ3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR3" s="58" t="inlineStr">
+      <c r="BR3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1113,12 +1116,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BQ4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1183,12 +1186,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BQ5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1248,12 +1251,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BQ6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1308,12 +1311,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BQ7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1390,12 +1393,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BQ8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1443,12 +1446,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BQ9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1496,12 +1499,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BQ10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1544,12 +1547,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BQ11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1602,8 +1605,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BQ13" s="42" t="n"/>
       <c r="BR13" s="42" t="n"/>
+      <c r="BS13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1659,12 +1662,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BQ14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR14" s="58" t="inlineStr">
+      <c r="BR14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1718,12 +1721,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BQ15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BR15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1810,12 +1813,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BQ16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR16" s="58" t="inlineStr">
+      <c r="BR16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1894,12 +1897,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BQ17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR17" s="58" t="inlineStr">
+      <c r="BR17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1962,12 +1965,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BQ18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR18" s="58" t="inlineStr">
+      <c r="BR18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2034,12 +2037,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BQ19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR19" s="71" t="inlineStr">
+      <c r="BR19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2103,12 +2106,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BQ20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR20" s="58" t="inlineStr">
+      <c r="BR20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2168,12 +2171,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BQ21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR21" s="71" t="inlineStr">
+      <c r="BR21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2235,12 +2238,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BQ22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR22" s="71" t="inlineStr">
+      <c r="BR22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2295,12 +2298,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BQ23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BR23" s="58" t="inlineStr">
+      <c r="BR23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BS23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-19
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BS41"/>
+  <dimension ref="A1:BT41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -936,14 +936,17 @@
         <v>46251.57309795139</v>
       </c>
       <c r="BQ1" s="56" t="n">
-        <v>46252.57610714522</v>
-      </c>
-      <c r="BR1" s="44" t="inlineStr">
+        <v>46252.57610714121</v>
+      </c>
+      <c r="BR1" s="56" t="n">
+        <v>46253.57716068693</v>
+      </c>
+      <c r="BS1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BS1" s="44" t="inlineStr">
+      <c r="BT1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -997,12 +1000,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BR2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS2" s="58" t="inlineStr">
+      <c r="BS2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1056,12 +1059,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BR3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS3" s="58" t="inlineStr">
+      <c r="BS3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1116,12 +1119,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BR4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1186,12 +1189,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BR5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1251,12 +1254,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BR6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1311,12 +1314,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BR7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1393,12 +1396,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BR8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1446,12 +1449,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BR9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1499,12 +1502,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BR10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1547,12 +1550,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BR11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1605,8 +1608,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BR13" s="42" t="n"/>
       <c r="BS13" s="42" t="n"/>
+      <c r="BT13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1662,12 +1665,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BR14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS14" s="58" t="inlineStr">
+      <c r="BS14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1721,12 +1724,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BR15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BS15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1813,12 +1816,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BR16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS16" s="58" t="inlineStr">
+      <c r="BS16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1897,12 +1900,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BR17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS17" s="58" t="inlineStr">
+      <c r="BS17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1965,12 +1968,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BR18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS18" s="58" t="inlineStr">
+      <c r="BS18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2037,12 +2040,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BR19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS19" s="71" t="inlineStr">
+      <c r="BS19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2106,12 +2109,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BR20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS20" s="58" t="inlineStr">
+      <c r="BS20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2171,12 +2174,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BR21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS21" s="71" t="inlineStr">
+      <c r="BS21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2238,12 +2241,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BR22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS22" s="71" t="inlineStr">
+      <c r="BS22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2298,12 +2301,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BR23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BS23" s="58" t="inlineStr">
+      <c r="BS23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BT23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-20
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BT41"/>
+  <dimension ref="A1:BU41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -939,14 +939,17 @@
         <v>46252.57610714121</v>
       </c>
       <c r="BR1" s="56" t="n">
-        <v>46253.57716068693</v>
-      </c>
-      <c r="BS1" s="44" t="inlineStr">
+        <v>46253.57716068287</v>
+      </c>
+      <c r="BS1" s="56" t="n">
+        <v>46254.57808369915</v>
+      </c>
+      <c r="BT1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BT1" s="44" t="inlineStr">
+      <c r="BU1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1000,12 +1003,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BS2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT2" s="58" t="inlineStr">
+      <c r="BT2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1059,12 +1062,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BS3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT3" s="58" t="inlineStr">
+      <c r="BT3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1119,12 +1122,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BS4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1189,12 +1192,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BS5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1254,12 +1257,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BS6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1314,12 +1317,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BS7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1396,12 +1399,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BS8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1449,12 +1452,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BS9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1502,12 +1505,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BS10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1550,12 +1553,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BS11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1608,8 +1611,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BS13" s="42" t="n"/>
       <c r="BT13" s="42" t="n"/>
+      <c r="BU13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1665,12 +1668,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BS14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT14" s="58" t="inlineStr">
+      <c r="BT14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1724,12 +1727,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BS15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BT15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1816,12 +1819,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BS16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT16" s="58" t="inlineStr">
+      <c r="BT16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1900,12 +1903,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BS17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT17" s="58" t="inlineStr">
+      <c r="BT17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1968,12 +1971,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BS18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT18" s="58" t="inlineStr">
+      <c r="BT18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2040,12 +2043,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BS19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT19" s="71" t="inlineStr">
+      <c r="BT19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2109,12 +2112,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BS20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT20" s="58" t="inlineStr">
+      <c r="BT20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2174,12 +2177,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BS21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT21" s="71" t="inlineStr">
+      <c r="BT21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2241,12 +2244,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BS22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT22" s="71" t="inlineStr">
+      <c r="BT22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2301,12 +2304,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BS23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BT23" s="58" t="inlineStr">
+      <c r="BT23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BU23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-21
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BU41"/>
+  <dimension ref="A1:BV41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -942,14 +942,17 @@
         <v>46253.57716068287</v>
       </c>
       <c r="BS1" s="56" t="n">
-        <v>46254.57808369915</v>
-      </c>
-      <c r="BT1" s="44" t="inlineStr">
+        <v>46254.5780837037</v>
+      </c>
+      <c r="BT1" s="56" t="n">
+        <v>46255.57755599295</v>
+      </c>
+      <c r="BU1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BU1" s="44" t="inlineStr">
+      <c r="BV1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1003,12 +1006,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BT2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU2" s="58" t="inlineStr">
+      <c r="BU2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1062,12 +1065,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BT3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU3" s="58" t="inlineStr">
+      <c r="BU3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1122,12 +1125,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BT4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1192,12 +1195,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BT5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1257,12 +1260,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BT6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1317,12 +1320,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BT7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1399,12 +1402,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BT8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1452,12 +1455,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BT9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1505,12 +1508,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BT10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1553,12 +1556,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BT11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1611,8 +1614,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BT13" s="42" t="n"/>
       <c r="BU13" s="42" t="n"/>
+      <c r="BV13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1668,12 +1671,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BT14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU14" s="58" t="inlineStr">
+      <c r="BU14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1727,12 +1730,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BT15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BU15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1819,12 +1822,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BT16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU16" s="58" t="inlineStr">
+      <c r="BU16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1903,12 +1906,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BT17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU17" s="58" t="inlineStr">
+      <c r="BU17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1971,12 +1974,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BT18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU18" s="58" t="inlineStr">
+      <c r="BU18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2043,12 +2046,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BT19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU19" s="71" t="inlineStr">
+      <c r="BU19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2112,12 +2115,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BT20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU20" s="58" t="inlineStr">
+      <c r="BU20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2177,12 +2180,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BT21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU21" s="71" t="inlineStr">
+      <c r="BU21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2244,12 +2247,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BT22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU22" s="71" t="inlineStr">
+      <c r="BU22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2304,12 +2307,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BT23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BU23" s="58" t="inlineStr">
+      <c r="BU23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BV23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-22
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BV41"/>
+  <dimension ref="A1:BW41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -945,14 +945,17 @@
         <v>46254.5780837037</v>
       </c>
       <c r="BT1" s="56" t="n">
-        <v>46255.57755599295</v>
-      </c>
-      <c r="BU1" s="44" t="inlineStr">
+        <v>46255.57755599537</v>
+      </c>
+      <c r="BU1" s="56" t="n">
+        <v>46256.56776790856</v>
+      </c>
+      <c r="BV1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BV1" s="44" t="inlineStr">
+      <c r="BW1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1006,12 +1009,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BU2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV2" s="58" t="inlineStr">
+      <c r="BV2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1065,12 +1068,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BU3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV3" s="58" t="inlineStr">
+      <c r="BV3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1125,12 +1128,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BU4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1195,12 +1198,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BU5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1260,12 +1263,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BU6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1320,12 +1323,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BU7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1402,12 +1405,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BU8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1455,12 +1458,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BU9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1508,12 +1511,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BU10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1556,12 +1559,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BU11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1614,8 +1617,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BU13" s="42" t="n"/>
       <c r="BV13" s="42" t="n"/>
+      <c r="BW13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1671,12 +1674,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BU14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV14" s="58" t="inlineStr">
+      <c r="BV14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1730,12 +1733,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BU15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BV15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1822,12 +1825,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BU16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV16" s="58" t="inlineStr">
+      <c r="BV16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1906,12 +1909,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BU17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV17" s="58" t="inlineStr">
+      <c r="BV17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1974,12 +1977,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BU18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV18" s="58" t="inlineStr">
+      <c r="BV18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2046,12 +2049,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BU19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV19" s="71" t="inlineStr">
+      <c r="BV19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2115,12 +2118,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BU20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV20" s="58" t="inlineStr">
+      <c r="BV20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2180,12 +2183,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BU21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV21" s="71" t="inlineStr">
+      <c r="BV21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2247,12 +2250,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BU22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV22" s="71" t="inlineStr">
+      <c r="BV22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2307,12 +2310,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BU23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BV23" s="58" t="inlineStr">
+      <c r="BV23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BW23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>